<commit_message>
DCF calibrado profesional: CapEx realista, escenarios estrechos y tesis GOOG/MSFT/CSU.TO
- Calibrar escenarios DCF: offsets ±15% growth, ±1pp WACC/margen, CapEx bear 1.15x/bull 0.90x
- Usar CapEx histórico real (no solo D&A) para proyecciones — bear case ahora ≈ precio de mercado
- Añadir capex_pct, sga_pct, rd_pct, da_pct, tax_rate al JSON de valoración por escenario
- Generar tesis completas: GOOG (infravalorada), MSFT (valor justo), CSU.TO (compra con convicción)
- Ratio bull/bear reducido de 2.72x a ~1.8x (dispersión profesional)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/valuations/AAPL/AAPL_modelo_valoracion.xlsx
+++ b/data/valuations/AAPL/AAPL_modelo_valoracion.xlsx
@@ -660,19 +660,19 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.2041</v>
+        <v>0.18055</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.18369</v>
+        <v>0.162495</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>0.16328</v>
+        <v>0.14444</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>0.14287</v>
+        <v>0.126385</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0.12246</v>
+        <v>0.10833</v>
       </c>
     </row>
     <row r="10">
@@ -682,19 +682,19 @@
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.1099</v>
+        <v>0.13345</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.09891</v>
+        <v>0.120105</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>0.08792</v>
+        <v>0.10676</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>0.07693</v>
+        <v>0.093415</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>0.06594</v>
+        <v>0.08007</v>
       </c>
     </row>
     <row r="11">
@@ -797,19 +797,19 @@
         </is>
       </c>
       <c r="G16" s="6" t="n">
-        <v>0.4713806851524051</v>
+        <v>0.4613806851524051</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0.4713806851524051</v>
+        <v>0.4613806851524051</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>0.4713806851524051</v>
+        <v>0.4613806851524051</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>0.4713806851524051</v>
+        <v>0.4613806851524051</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>0.4713806851524051</v>
+        <v>0.4613806851524051</v>
       </c>
     </row>
     <row r="17">
@@ -819,19 +819,19 @@
         </is>
       </c>
       <c r="G17" s="6" t="n">
-        <v>0.4313806851524051</v>
+        <v>0.4413806851524051</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>0.4313806851524051</v>
+        <v>0.4413806851524051</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>0.4313806851524051</v>
+        <v>0.4413806851524051</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>0.4313806851524051</v>
+        <v>0.4413806851524051</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>0.4313806851524051</v>
+        <v>0.4413806851524051</v>
       </c>
     </row>
     <row r="18">
@@ -890,19 +890,19 @@
         </is>
       </c>
       <c r="G21" s="6" t="n">
-        <v>0.05543668517974536</v>
+        <v>0.06043668517974537</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>0.05543668517974536</v>
+        <v>0.06043668517974537</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.05543668517974536</v>
+        <v>0.06043668517974537</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>0.05543668517974536</v>
+        <v>0.06043668517974537</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>0.05543668517974536</v>
+        <v>0.06043668517974537</v>
       </c>
     </row>
     <row r="22">
@@ -912,19 +912,19 @@
         </is>
       </c>
       <c r="G22" s="6" t="n">
-        <v>0.07543668517974536</v>
+        <v>0.07043668517974537</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.07543668517974536</v>
+        <v>0.07043668517974537</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>0.07543668517974536</v>
+        <v>0.07043668517974537</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.07543668517974536</v>
+        <v>0.07043668517974537</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>0.07543668517974536</v>
+        <v>0.07043668517974537</v>
       </c>
     </row>
     <row r="23">
@@ -1005,19 +1005,19 @@
         </is>
       </c>
       <c r="G27" s="6" t="n">
-        <v>0.08196605173960779</v>
+        <v>0.07696605173960779</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>0.08196605173960779</v>
+        <v>0.07696605173960779</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>0.08196605173960779</v>
+        <v>0.07696605173960779</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>0.08196605173960779</v>
+        <v>0.07696605173960779</v>
       </c>
       <c r="K27" s="6" t="n">
-        <v>0.08196605173960779</v>
+        <v>0.07696605173960779</v>
       </c>
     </row>
     <row r="28">
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>0.1248</v>
+        <v>0.1148</v>
       </c>
     </row>
     <row r="38">
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="C42" s="9" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="43">
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="F2" s="16" t="n">
-        <v>259.88</v>
+        <v>247.99</v>
       </c>
     </row>
     <row r="4">
@@ -3698,7 +3698,7 @@
         </is>
       </c>
       <c r="C34" s="20">
-        <f>C33/259.88-1</f>
+        <f>C33/247.99-1</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Reescritura de 24 tesis + mejoras quality gates + paso interpretativo obligatorio
- Fix bug analyst.py: sec_audit no se pasaba a _build_valuation_summary
- quality_gates.py: 3 checks nuevos (compresión múltiplo, gap consenso, valoración extrema→CRITICAL)
- thesis_reviewer.py: bear check siempre activo, gap consenso, check fuentes primarias
- financial_data.py: TV multiples auto-ajustados si EV/EBITDA > TV×5 (ej: Tesla 12x→24x)
- Borrado dashboard.py antiguo (pendiente recrear)
- 24 tesis actualizadas con datos 28/03/2026
- 4 tesis con paso interpretativo completo (AAPL, AMZN, CSU_TO, DE): 10-K + noticias + criterio
- Limpieza de tickers obsoletos (1ZG_F, 31L_SG, AFM_V, NWL, NYY_F, SANA)
- Nuevo: MCD, sec_parser.py, historiales de valoración

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/valuations/AAPL/AAPL_modelo_valoracion.xlsx
+++ b/data/valuations/AAPL/AAPL_modelo_valoracion.xlsx
@@ -1076,19 +1076,19 @@
         </is>
       </c>
       <c r="G31" s="6" t="n">
-        <v>0.02761485036770544</v>
+        <v>0.02787367975059465</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>0.02761485036770544</v>
+        <v>0.02787367975059465</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>0.02761485036770544</v>
+        <v>0.02787367975059465</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>0.02761485036770544</v>
+        <v>0.02787367975059465</v>
       </c>
       <c r="K31" s="6" t="n">
-        <v>0.02761485036770544</v>
+        <v>0.02787367975059465</v>
       </c>
     </row>
     <row r="32">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>0.1048</v>
+        <v>0.1051</v>
       </c>
     </row>
     <row r="36">
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>0.09480000000000001</v>
+        <v>0.0951</v>
       </c>
     </row>
     <row r="37">
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>0.1148</v>
+        <v>0.1151</v>
       </c>
     </row>
     <row r="38">
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="F2" s="16" t="n">
-        <v>247.99</v>
+        <v>248.8</v>
       </c>
     </row>
     <row r="4">
@@ -3584,7 +3584,7 @@
         </is>
       </c>
       <c r="K21" s="8">
-        <f>K12*$C$16</f>
+        <f>K8*$C$16</f>
         <v/>
       </c>
     </row>
@@ -3698,7 +3698,7 @@
         </is>
       </c>
       <c r="C34" s="20">
-        <f>C33/247.99-1</f>
+        <f>C33/248.8-1</f>
         <v/>
       </c>
     </row>
@@ -3753,176 +3753,176 @@
     </row>
     <row r="39">
       <c r="A39" s="21" t="n">
-        <v>0.07480000000000001</v>
+        <v>0.0751</v>
       </c>
       <c r="C39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$12*15/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*15/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$12*17/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*17/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$12*19/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*19/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$12*21/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*21/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$12*23/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*23/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="21" t="n">
-        <v>0.0848</v>
+        <v>0.0851</v>
       </c>
       <c r="C40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$12*15/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*15/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$12*17/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*17/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$12*19/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*19/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$12*21/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*21/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$12*23/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*23/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="n">
-        <v>0.09480000000000001</v>
+        <v>0.0951</v>
       </c>
       <c r="C41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$12*15/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*15/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$12*17/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*17/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$12*19/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*19/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$12*21/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*21/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$12*23/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*23/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="21" t="n">
-        <v>0.1048</v>
+        <v>0.1051</v>
       </c>
       <c r="C42" s="22">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$12*15/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*15/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D42" s="22">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$12*17/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*17/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E42" s="23">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$12*19/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*19/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F42" s="22">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$12*21/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*21/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G42" s="22">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$12*23/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*23/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="21" t="n">
-        <v>0.1148</v>
+        <v>0.1151</v>
       </c>
       <c r="C43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$12*15/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*15/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$12*17/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*17/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$12*19/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*19/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$12*21/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*21/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$12*23/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*23/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="21" t="n">
-        <v>0.1248</v>
+        <v>0.1251</v>
       </c>
       <c r="C44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$12*15/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*15/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$12*17/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*17/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$12*19/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*19/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$12*21/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*21/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$12*23/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*23/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="n">
-        <v>0.1348</v>
+        <v>0.1351</v>
       </c>
       <c r="C45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$12*15/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*15/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$12*17/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*17/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$12*19/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*19/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$12*21/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*21/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$12*23/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*23/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización masiva de valoraciones abril 2026 y mejoras de tools
- Reescritura de tesis y valoraciones para 26 tickers con datos actualizados
- Snapshots históricos 20260404 para tracking de evolución
- Nuevos tickers: ASTS, MAU_PA, OXY
- Eliminación de ITX (datos obsoletos)
- Mejoras en financial_data.py, check_inbox.py, message_queue.py, telegram_bot.py
- Artículos y tracker de reescritura de tesis

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/valuations/AAPL/AAPL_modelo_valoracion.xlsx
+++ b/data/valuations/AAPL/AAPL_modelo_valoracion.xlsx
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>0.1051</v>
+        <v>0.1046</v>
       </c>
     </row>
     <row r="36">
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>0.0951</v>
+        <v>0.0946</v>
       </c>
     </row>
     <row r="37">
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>0.1151</v>
+        <v>0.1146</v>
       </c>
     </row>
     <row r="38">
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="F2" s="16" t="n">
-        <v>248.8</v>
+        <v>255.92</v>
       </c>
     </row>
     <row r="4">
@@ -3698,7 +3698,7 @@
         </is>
       </c>
       <c r="C34" s="20">
-        <f>C33/248.8-1</f>
+        <f>C33/255.92-1</f>
         <v/>
       </c>
     </row>
@@ -3753,7 +3753,7 @@
     </row>
     <row r="39">
       <c r="A39" s="21" t="n">
-        <v>0.0751</v>
+        <v>0.0746</v>
       </c>
       <c r="C39" s="22">
         <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*15/(1+$A$39)^5+$C$29)/$C$32</f>
@@ -3778,7 +3778,7 @@
     </row>
     <row r="40">
       <c r="A40" s="21" t="n">
-        <v>0.0851</v>
+        <v>0.08459999999999999</v>
       </c>
       <c r="C40" s="22">
         <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*15/(1+$A$40)^5+$C$29)/$C$32</f>
@@ -3803,7 +3803,7 @@
     </row>
     <row r="41">
       <c r="A41" s="21" t="n">
-        <v>0.0951</v>
+        <v>0.0946</v>
       </c>
       <c r="C41" s="22">
         <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*15/(1+$A$41)^5+$C$29)/$C$32</f>
@@ -3828,7 +3828,7 @@
     </row>
     <row r="42">
       <c r="A42" s="21" t="n">
-        <v>0.1051</v>
+        <v>0.1046</v>
       </c>
       <c r="C42" s="22">
         <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*15/(1+$A$42)^5+$C$29)/$C$32</f>
@@ -3853,7 +3853,7 @@
     </row>
     <row r="43">
       <c r="A43" s="21" t="n">
-        <v>0.1151</v>
+        <v>0.1146</v>
       </c>
       <c r="C43" s="22">
         <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*15/(1+$A$43)^5+$C$29)/$C$32</f>
@@ -3878,7 +3878,7 @@
     </row>
     <row r="44">
       <c r="A44" s="21" t="n">
-        <v>0.1251</v>
+        <v>0.1246</v>
       </c>
       <c r="C44" s="22">
         <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*15/(1+$A$44)^5+$C$29)/$C$32</f>
@@ -3903,7 +3903,7 @@
     </row>
     <row r="45">
       <c r="A45" s="21" t="n">
-        <v>0.1351</v>
+        <v>0.1346</v>
       </c>
       <c r="C45" s="22">
         <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*15/(1+$A$45)^5+$C$29)/$C$32</f>

</xml_diff>

<commit_message>
Punto de retorno estable: sistema completo antes del rediseño
Estado consolidado del sistema investment-agents tal como funciona hoy,
guardado como línea base por si el rediseño posterior no convence.

Incluye:
- Pipeline Python (recolección de datos) + skills de Claude Code (interpretación)
- Bot de Telegram multiusuario (Kiko + 2 amigos) vía cola + /loop, sin API
- Últimas correcciones ya integradas: review gate programático,
  fix parser SEC (scale/sign XBRL), fix filas Excel DCF, escrituras atómicas
- Valoraciones y tesis vigentes en data/valuations/

Para volver a este estado: git reset --hard pre-rediseno-2026

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/valuations/AAPL/AAPL_modelo_valoracion.xlsx
+++ b/data/valuations/AAPL/AAPL_modelo_valoracion.xlsx
@@ -638,19 +638,19 @@
         </is>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.157</v>
+        <v>0.06</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.1413</v>
+        <v>0.05</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>0.1256</v>
+        <v>0.04</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>0.1099</v>
+        <v>0.04</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0.09419999999999999</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="9">
@@ -660,19 +660,19 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.18055</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.162495</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>0.14444</v>
+        <v>0.055</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>0.126385</v>
+        <v>0.05</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0.10833</v>
+        <v>0.045</v>
       </c>
     </row>
     <row r="10">
@@ -682,19 +682,19 @@
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.13345</v>
+        <v>0.03</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.120105</v>
+        <v>0</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>0.10676</v>
+        <v>-0.02</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>0.093415</v>
+        <v>0.01</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>0.08007</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="11">
@@ -775,19 +775,19 @@
         </is>
       </c>
       <c r="G15" s="6" t="n">
-        <v>0.4513806851524051</v>
+        <v>0.465</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>0.4513806851524051</v>
+        <v>0.465</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>0.4513806851524051</v>
+        <v>0.465</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>0.4513806851524051</v>
+        <v>0.465</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>0.4513806851524051</v>
+        <v>0.465</v>
       </c>
     </row>
     <row r="16">
@@ -797,19 +797,19 @@
         </is>
       </c>
       <c r="G16" s="6" t="n">
-        <v>0.4613806851524051</v>
+        <v>0.475</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0.4613806851524051</v>
+        <v>0.475</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>0.4613806851524051</v>
+        <v>0.475</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>0.4613806851524051</v>
+        <v>0.475</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>0.4613806851524051</v>
+        <v>0.475</v>
       </c>
     </row>
     <row r="17">
@@ -819,19 +819,19 @@
         </is>
       </c>
       <c r="G17" s="6" t="n">
-        <v>0.4413806851524051</v>
+        <v>0.435</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>0.4413806851524051</v>
+        <v>0.435</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>0.4413806851524051</v>
+        <v>0.435</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>0.4413806851524051</v>
+        <v>0.435</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>0.4413806851524051</v>
+        <v>0.435</v>
       </c>
     </row>
     <row r="18">
@@ -868,19 +868,19 @@
         </is>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0.06543668517974537</v>
+        <v>0.065</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>0.06543668517974537</v>
+        <v>0.065</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.06543668517974537</v>
+        <v>0.065</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>0.06543668517974537</v>
+        <v>0.065</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>0.06543668517974537</v>
+        <v>0.065</v>
       </c>
     </row>
     <row r="21">
@@ -890,19 +890,19 @@
         </is>
       </c>
       <c r="G21" s="6" t="n">
-        <v>0.06043668517974537</v>
+        <v>0.063</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>0.06043668517974537</v>
+        <v>0.063</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.06043668517974537</v>
+        <v>0.063</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>0.06043668517974537</v>
+        <v>0.063</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>0.06043668517974537</v>
+        <v>0.063</v>
       </c>
     </row>
     <row r="22">
@@ -912,19 +912,19 @@
         </is>
       </c>
       <c r="G22" s="6" t="n">
-        <v>0.07043668517974537</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.07043668517974537</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>0.07043668517974537</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.07043668517974537</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>0.07043668517974537</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="23">
@@ -961,19 +961,19 @@
         </is>
       </c>
       <c r="G25" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.08</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.08</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.08</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.08</v>
       </c>
       <c r="K25" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="26">
@@ -983,19 +983,19 @@
         </is>
       </c>
       <c r="G26" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.078</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.078</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.078</v>
       </c>
       <c r="J26" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.078</v>
       </c>
       <c r="K26" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.078</v>
       </c>
     </row>
     <row r="27">
@@ -1005,19 +1005,19 @@
         </is>
       </c>
       <c r="G27" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.08</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.08</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.08</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.08</v>
       </c>
       <c r="K27" s="6" t="n">
-        <v>0.07696605173960779</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="28">
@@ -1054,19 +1054,19 @@
         </is>
       </c>
       <c r="G30" s="6" t="n">
-        <v>0.02889761166940512</v>
+        <v>0.029</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0.02889761166940512</v>
+        <v>0.029</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>0.02889761166940512</v>
+        <v>0.029</v>
       </c>
       <c r="J30" s="6" t="n">
-        <v>0.02889761166940512</v>
+        <v>0.029</v>
       </c>
       <c r="K30" s="6" t="n">
-        <v>0.02889761166940512</v>
+        <v>0.029</v>
       </c>
     </row>
     <row r="31">
@@ -1076,19 +1076,19 @@
         </is>
       </c>
       <c r="G31" s="6" t="n">
-        <v>0.02787367975059465</v>
+        <v>0.03</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>0.02787367975059465</v>
+        <v>0.03</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>0.02787367975059465</v>
+        <v>0.03</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>0.02787367975059465</v>
+        <v>0.03</v>
       </c>
       <c r="K31" s="6" t="n">
-        <v>0.02787367975059465</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="32">
@@ -1098,19 +1098,19 @@
         </is>
       </c>
       <c r="G32" s="6" t="n">
-        <v>0.1763042098965495</v>
+        <v>0.176</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0.1763042098965495</v>
+        <v>0.176</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>0.1763042098965495</v>
+        <v>0.176</v>
       </c>
       <c r="J32" s="6" t="n">
-        <v>0.1763042098965495</v>
+        <v>0.176</v>
       </c>
       <c r="K32" s="6" t="n">
-        <v>0.1763042098965495</v>
+        <v>0.176</v>
       </c>
     </row>
     <row r="34">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>0.1046</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="36">
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>0.0946</v>
+        <v>0.095</v>
       </c>
     </row>
     <row r="37">
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>0.1146</v>
+        <v>0.105</v>
       </c>
     </row>
     <row r="38">
@@ -1178,7 +1178,7 @@
         </is>
       </c>
       <c r="C40" s="9" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41">
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="C41" s="9" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="42">
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="C42" s="9" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43">
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="F2" s="16" t="n">
-        <v>255.92</v>
+        <v>300.23</v>
       </c>
     </row>
     <row r="4">
@@ -3677,7 +3677,7 @@
         </is>
       </c>
       <c r="C32" s="18" t="n">
-        <v>14681.14</v>
+        <v>14687.356</v>
       </c>
     </row>
     <row r="33">
@@ -3698,7 +3698,7 @@
         </is>
       </c>
       <c r="C34" s="20">
-        <f>C33/255.92-1</f>
+        <f>C33/300.23-1</f>
         <v/>
       </c>
     </row>
@@ -3727,202 +3727,202 @@
       </c>
       <c r="C38" s="1" t="inlineStr">
         <is>
-          <t>15x</t>
+          <t>16x</t>
         </is>
       </c>
       <c r="D38" s="1" t="inlineStr">
         <is>
-          <t>17x</t>
+          <t>18x</t>
         </is>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>19x</t>
+          <t>20x</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>21x</t>
+          <t>22x</t>
         </is>
       </c>
       <c r="G38" s="1" t="inlineStr">
         <is>
-          <t>23x</t>
+          <t>24x</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="21" t="n">
-        <v>0.0746</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*15/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*16/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*17/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*18/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*19/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*20/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*21/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*22/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*23/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*24/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="21" t="n">
-        <v>0.08459999999999999</v>
+        <v>0.08</v>
       </c>
       <c r="C40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*15/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*16/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*17/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*18/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*19/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*20/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*21/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*22/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*23/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*24/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="n">
-        <v>0.0946</v>
+        <v>0.09000000000000001</v>
       </c>
       <c r="C41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*15/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*16/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*17/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*18/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*19/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*20/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*21/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*22/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*23/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*24/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="21" t="n">
-        <v>0.1046</v>
+        <v>0.1</v>
       </c>
       <c r="C42" s="22">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*15/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*16/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D42" s="22">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*17/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*18/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E42" s="23">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*19/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*20/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F42" s="22">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*21/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*22/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G42" s="22">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*23/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*24/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="21" t="n">
-        <v>0.1146</v>
+        <v>0.11</v>
       </c>
       <c r="C43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*15/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*16/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*17/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*18/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*19/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*20/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*21/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*22/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*23/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*24/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="21" t="n">
-        <v>0.1246</v>
+        <v>0.12</v>
       </c>
       <c r="C44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*15/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*16/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*17/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*18/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*19/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*20/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*21/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*22/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*23/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*24/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="n">
-        <v>0.1346</v>
+        <v>0.13</v>
       </c>
       <c r="C45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*15/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*16/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*17/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*18/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*19/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*20/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*21/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*22/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*23/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*24/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>

</xml_diff>